<commit_message>
Use formatted DX schedule template for export
</commit_message>
<xml_diff>
--- a/data/dx-selection-template.xlsx
+++ b/data/dx-selection-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6250AAF-590A-469A-9995-169DEA3ED08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501667C8-4D15-423C-AF37-2B9309A6A30B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -727,7 +727,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -1364,7 +1364,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1427,10 +1427,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1569,104 +1569,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1702,7 +1604,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1711,11 +1625,97 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1798,8 +1798,8 @@
     <xdr:to>
       <xdr:col>30</xdr:col>
       <xdr:colOff>463628</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>184171</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>3357</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2383,173 +2383,173 @@
     </row>
     <row r="11" spans="2:41" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="2:41" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="117" t="s">
+      <c r="B12" s="87" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="118"/>
-      <c r="D12" s="118"/>
-      <c r="E12" s="118"/>
-      <c r="F12" s="118"/>
-      <c r="G12" s="119"/>
-      <c r="H12" s="125" t="s">
+      <c r="C12" s="88"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="88"/>
+      <c r="F12" s="88"/>
+      <c r="G12" s="89"/>
+      <c r="H12" s="95" t="s">
         <v>78</v>
       </c>
-      <c r="I12" s="125"/>
-      <c r="J12" s="125"/>
-      <c r="K12" s="125"/>
-      <c r="L12" s="125"/>
-      <c r="M12" s="125"/>
-      <c r="N12" s="125"/>
-      <c r="O12" s="125"/>
-      <c r="P12" s="125"/>
-      <c r="Q12" s="125"/>
-      <c r="R12" s="125"/>
-      <c r="S12" s="125"/>
-      <c r="T12" s="125"/>
-      <c r="U12" s="125"/>
-      <c r="V12" s="125"/>
-      <c r="W12" s="125"/>
-      <c r="X12" s="125"/>
-      <c r="Y12" s="125"/>
-      <c r="Z12" s="125"/>
-      <c r="AA12" s="125"/>
-      <c r="AB12" s="125"/>
-      <c r="AC12" s="125"/>
-      <c r="AD12" s="125"/>
-      <c r="AE12" s="126"/>
+      <c r="I12" s="95"/>
+      <c r="J12" s="95"/>
+      <c r="K12" s="95"/>
+      <c r="L12" s="95"/>
+      <c r="M12" s="95"/>
+      <c r="N12" s="95"/>
+      <c r="O12" s="95"/>
+      <c r="P12" s="95"/>
+      <c r="Q12" s="95"/>
+      <c r="R12" s="95"/>
+      <c r="S12" s="95"/>
+      <c r="T12" s="95"/>
+      <c r="U12" s="95"/>
+      <c r="V12" s="95"/>
+      <c r="W12" s="95"/>
+      <c r="X12" s="95"/>
+      <c r="Y12" s="95"/>
+      <c r="Z12" s="95"/>
+      <c r="AA12" s="95"/>
+      <c r="AB12" s="95"/>
+      <c r="AC12" s="95"/>
+      <c r="AD12" s="95"/>
+      <c r="AE12" s="96"/>
     </row>
     <row r="13" spans="2:41" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="120" t="s">
+      <c r="B13" s="90" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="122" t="s">
+      <c r="C13" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="122" t="s">
+      <c r="D13" s="92" t="s">
         <v>75</v>
       </c>
-      <c r="E13" s="111" t="s">
+      <c r="E13" s="108" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="111" t="s">
+      <c r="F13" s="108" t="s">
         <v>77</v>
       </c>
-      <c r="G13" s="114" t="s">
+      <c r="G13" s="111" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="106" t="s">
+      <c r="H13" s="115" t="s">
         <v>98</v>
       </c>
-      <c r="I13" s="109" t="s">
+      <c r="I13" s="100" t="s">
         <v>79</v>
       </c>
-      <c r="J13" s="109" t="s">
+      <c r="J13" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="109" t="s">
+      <c r="K13" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="L13" s="109" t="s">
+      <c r="L13" s="100" t="s">
         <v>17</v>
       </c>
-      <c r="M13" s="110" t="s">
+      <c r="M13" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="N13" s="110"/>
-      <c r="O13" s="128" t="s">
+      <c r="N13" s="97"/>
+      <c r="O13" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="P13" s="128"/>
+      <c r="P13" s="102"/>
       <c r="Q13" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="R13" s="129" t="s">
+      <c r="R13" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="S13" s="130" t="s">
+      <c r="S13" s="105" t="s">
         <v>70</v>
       </c>
-      <c r="T13" s="131"/>
-      <c r="U13" s="110" t="s">
+      <c r="T13" s="106"/>
+      <c r="U13" s="97" t="s">
         <v>25</v>
       </c>
-      <c r="V13" s="110" t="s">
+      <c r="V13" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="W13" s="110" t="s">
+      <c r="W13" s="97" t="s">
         <v>5</v>
       </c>
-      <c r="X13" s="110" t="s">
+      <c r="X13" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="Y13" s="110"/>
-      <c r="Z13" s="110"/>
-      <c r="AA13" s="110" t="s">
+      <c r="Y13" s="97"/>
+      <c r="Z13" s="97"/>
+      <c r="AA13" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="AB13" s="110"/>
-      <c r="AC13" s="110"/>
-      <c r="AD13" s="110" t="s">
+      <c r="AB13" s="97"/>
+      <c r="AC13" s="97"/>
+      <c r="AD13" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="AE13" s="127"/>
-      <c r="AG13" s="105" t="s">
+      <c r="AE13" s="98"/>
+      <c r="AG13" s="114" t="s">
         <v>99</v>
       </c>
-      <c r="AH13" s="105"/>
-      <c r="AI13" s="105"/>
-      <c r="AJ13" s="105"/>
-      <c r="AK13" s="105"/>
-      <c r="AL13" s="105"/>
-      <c r="AM13" s="105"/>
-      <c r="AN13" s="105"/>
-      <c r="AO13" s="105"/>
+      <c r="AH13" s="114"/>
+      <c r="AI13" s="114"/>
+      <c r="AJ13" s="114"/>
+      <c r="AK13" s="114"/>
+      <c r="AL13" s="114"/>
+      <c r="AM13" s="114"/>
+      <c r="AN13" s="114"/>
+      <c r="AO13" s="114"/>
     </row>
     <row r="14" spans="2:41" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="121"/>
-      <c r="C14" s="123"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="112"/>
-      <c r="F14" s="112"/>
-      <c r="G14" s="115"/>
-      <c r="H14" s="107"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="95"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="90" t="s">
+      <c r="B14" s="91"/>
+      <c r="C14" s="93"/>
+      <c r="D14" s="93"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="112"/>
+      <c r="H14" s="116"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="101"/>
+      <c r="K14" s="101"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="N14" s="90"/>
-      <c r="O14" s="90" t="s">
+      <c r="N14" s="99"/>
+      <c r="O14" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="P14" s="90" t="s">
+      <c r="P14" s="99" t="s">
         <v>9</v>
       </c>
-      <c r="Q14" s="90" t="s">
+      <c r="Q14" s="99" t="s">
         <v>10</v>
       </c>
-      <c r="R14" s="94"/>
-      <c r="S14" s="92" t="s">
+      <c r="R14" s="104"/>
+      <c r="S14" s="107" t="s">
         <v>71</v>
       </c>
-      <c r="T14" s="95" t="s">
+      <c r="T14" s="101" t="s">
         <v>72</v>
       </c>
-      <c r="U14" s="90"/>
-      <c r="V14" s="90"/>
-      <c r="W14" s="90"/>
-      <c r="X14" s="90" t="s">
+      <c r="U14" s="99"/>
+      <c r="V14" s="99"/>
+      <c r="W14" s="99"/>
+      <c r="X14" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="Y14" s="90"/>
-      <c r="Z14" s="90"/>
-      <c r="AA14" s="90" t="s">
+      <c r="Y14" s="99"/>
+      <c r="Z14" s="99"/>
+      <c r="AA14" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="AB14" s="90"/>
-      <c r="AC14" s="90"/>
+      <c r="AB14" s="99"/>
+      <c r="AC14" s="99"/>
       <c r="AD14" s="13" t="s">
         <v>16</v>
       </c>
@@ -2558,34 +2558,34 @@
       </c>
     </row>
     <row r="15" spans="2:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="121"/>
-      <c r="C15" s="124"/>
-      <c r="D15" s="124"/>
-      <c r="E15" s="113"/>
-      <c r="F15" s="113"/>
-      <c r="G15" s="116"/>
-      <c r="H15" s="108"/>
-      <c r="I15" s="96"/>
-      <c r="J15" s="95"/>
-      <c r="K15" s="95"/>
-      <c r="L15" s="95"/>
+      <c r="B15" s="91"/>
+      <c r="C15" s="94"/>
+      <c r="D15" s="94"/>
+      <c r="E15" s="110"/>
+      <c r="F15" s="110"/>
+      <c r="G15" s="113"/>
+      <c r="H15" s="117"/>
+      <c r="I15" s="118"/>
+      <c r="J15" s="101"/>
+      <c r="K15" s="101"/>
+      <c r="L15" s="101"/>
       <c r="M15" s="15" t="s">
         <v>16</v>
       </c>
       <c r="N15" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="O15" s="92"/>
-      <c r="P15" s="92"/>
-      <c r="Q15" s="92"/>
-      <c r="R15" s="94"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
+      <c r="O15" s="107"/>
+      <c r="P15" s="107"/>
+      <c r="Q15" s="107"/>
+      <c r="R15" s="104"/>
+      <c r="S15" s="101"/>
+      <c r="T15" s="101"/>
       <c r="U15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="V15" s="92"/>
-      <c r="W15" s="92"/>
+      <c r="V15" s="107"/>
+      <c r="W15" s="107"/>
       <c r="X15" s="15" t="s">
         <v>19</v>
       </c>
@@ -23690,6 +23690,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="AG13:AO13"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="S14:S15"/>
+    <mergeCell ref="T14:T15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="V13:V15"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="M14:N14"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="C13:C15"/>
@@ -23706,22 +23722,6 @@
     <mergeCell ref="X13:Z13"/>
     <mergeCell ref="AA13:AC13"/>
     <mergeCell ref="X14:Z14"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="G13:G15"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="AG13:AO13"/>
-    <mergeCell ref="H13:H15"/>
-    <mergeCell ref="S14:S15"/>
-    <mergeCell ref="T14:T15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="V13:V15"/>
-    <mergeCell ref="O14:O15"/>
-    <mergeCell ref="J13:J15"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
@@ -23783,135 +23783,135 @@
   <sheetData>
     <row r="1" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="127" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
-      <c r="L2" s="88"/>
-      <c r="M2" s="88"/>
-      <c r="N2" s="88"/>
-      <c r="O2" s="88"/>
-      <c r="P2" s="88"/>
-      <c r="Q2" s="88"/>
-      <c r="R2" s="88"/>
-      <c r="S2" s="88"/>
-      <c r="T2" s="88"/>
-      <c r="U2" s="88"/>
-      <c r="V2" s="88"/>
-      <c r="W2" s="88"/>
-      <c r="X2" s="88"/>
-      <c r="Y2" s="89"/>
+      <c r="B2" s="128"/>
+      <c r="C2" s="128"/>
+      <c r="D2" s="128"/>
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="128"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="128"/>
+      <c r="J2" s="128"/>
+      <c r="K2" s="128"/>
+      <c r="L2" s="128"/>
+      <c r="M2" s="128"/>
+      <c r="N2" s="128"/>
+      <c r="O2" s="128"/>
+      <c r="P2" s="128"/>
+      <c r="Q2" s="128"/>
+      <c r="R2" s="128"/>
+      <c r="S2" s="128"/>
+      <c r="T2" s="128"/>
+      <c r="U2" s="128"/>
+      <c r="V2" s="128"/>
+      <c r="W2" s="128"/>
+      <c r="X2" s="128"/>
+      <c r="Y2" s="129"/>
     </row>
     <row r="3" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="122" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="101"/>
+      <c r="B3" s="123"/>
       <c r="C3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="92" t="s">
+      <c r="D3" s="107" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="92" t="s">
+      <c r="E3" s="107" t="s">
         <v>45</v>
       </c>
-      <c r="F3" s="92" t="s">
+      <c r="F3" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="90" t="s">
+      <c r="G3" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="90"/>
-      <c r="I3" s="102" t="s">
+      <c r="H3" s="99"/>
+      <c r="I3" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="102"/>
+      <c r="J3" s="124"/>
       <c r="K3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="93" t="s">
+      <c r="L3" s="131" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="103" t="s">
+      <c r="M3" s="125" t="s">
         <v>70</v>
       </c>
-      <c r="N3" s="104"/>
-      <c r="O3" s="90" t="s">
+      <c r="N3" s="126"/>
+      <c r="O3" s="99" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="90" t="s">
+      <c r="P3" s="99" t="s">
         <v>4</v>
       </c>
-      <c r="Q3" s="90" t="s">
+      <c r="Q3" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="R3" s="90" t="s">
+      <c r="R3" s="99" t="s">
         <v>6</v>
       </c>
-      <c r="S3" s="90"/>
-      <c r="T3" s="90"/>
-      <c r="U3" s="90" t="s">
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
+      <c r="U3" s="99" t="s">
         <v>6</v>
       </c>
-      <c r="V3" s="90"/>
-      <c r="W3" s="90"/>
-      <c r="X3" s="90" t="s">
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99" t="s">
         <v>7</v>
       </c>
-      <c r="Y3" s="91"/>
+      <c r="Y3" s="130"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A4" s="100"/>
-      <c r="B4" s="101"/>
-      <c r="C4" s="90" t="s">
+      <c r="A4" s="122"/>
+      <c r="B4" s="123"/>
+      <c r="C4" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="90" t="s">
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90" t="s">
+      <c r="H4" s="99"/>
+      <c r="I4" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="90" t="s">
+      <c r="J4" s="99" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="90" t="s">
+      <c r="K4" s="99" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="94"/>
-      <c r="M4" s="92" t="s">
+      <c r="L4" s="104"/>
+      <c r="M4" s="107" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="95" t="s">
+      <c r="N4" s="101" t="s">
         <v>72</v>
       </c>
-      <c r="O4" s="90"/>
-      <c r="P4" s="90"/>
-      <c r="Q4" s="90"/>
-      <c r="R4" s="90" t="s">
+      <c r="O4" s="99"/>
+      <c r="P4" s="99"/>
+      <c r="Q4" s="99"/>
+      <c r="R4" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="S4" s="90"/>
-      <c r="T4" s="90"/>
-      <c r="U4" s="90" t="s">
+      <c r="S4" s="99"/>
+      <c r="T4" s="99"/>
+      <c r="U4" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="V4" s="90"/>
-      <c r="W4" s="90"/>
+      <c r="V4" s="99"/>
+      <c r="W4" s="99"/>
       <c r="X4" s="13" t="s">
         <v>16</v>
       </c>
@@ -23924,27 +23924,27 @@
         <v>29</v>
       </c>
       <c r="B5" s="17"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="96"/>
-      <c r="E5" s="96"/>
-      <c r="F5" s="96"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
       <c r="G5" s="15" t="s">
         <v>16</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="92"/>
-      <c r="J5" s="92"/>
-      <c r="K5" s="92"/>
-      <c r="L5" s="94"/>
-      <c r="M5" s="96"/>
-      <c r="N5" s="95"/>
+      <c r="I5" s="107"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="107"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="118"/>
+      <c r="N5" s="101"/>
       <c r="O5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="92"/>
-      <c r="Q5" s="92"/>
+      <c r="P5" s="107"/>
+      <c r="Q5" s="107"/>
       <c r="R5" s="15" t="s">
         <v>19</v>
       </c>
@@ -23971,7 +23971,7 @@
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A6" s="97" t="s">
+      <c r="A6" s="119" t="s">
         <v>38</v>
       </c>
       <c r="B6" s="9" t="s">
@@ -24048,7 +24048,7 @@
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A7" s="98"/>
+      <c r="A7" s="120"/>
       <c r="B7" s="2" t="s">
         <v>39</v>
       </c>
@@ -24123,7 +24123,7 @@
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A8" s="98"/>
+      <c r="A8" s="120"/>
       <c r="B8" s="2" t="s">
         <v>39</v>
       </c>
@@ -24198,7 +24198,7 @@
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A9" s="98"/>
+      <c r="A9" s="120"/>
       <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
@@ -24273,7 +24273,7 @@
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A10" s="98"/>
+      <c r="A10" s="120"/>
       <c r="B10" s="2" t="s">
         <v>39</v>
       </c>
@@ -24348,7 +24348,7 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="98"/>
+      <c r="A11" s="120"/>
       <c r="B11" s="4" t="s">
         <v>39</v>
       </c>
@@ -24423,7 +24423,7 @@
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A12" s="98"/>
+      <c r="A12" s="120"/>
       <c r="B12" s="9" t="s">
         <v>40</v>
       </c>
@@ -24498,7 +24498,7 @@
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A13" s="98"/>
+      <c r="A13" s="120"/>
       <c r="B13" s="2" t="s">
         <v>40</v>
       </c>
@@ -24573,7 +24573,7 @@
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A14" s="98"/>
+      <c r="A14" s="120"/>
       <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
@@ -24648,7 +24648,7 @@
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A15" s="98"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
@@ -24723,7 +24723,7 @@
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A16" s="98"/>
+      <c r="A16" s="120"/>
       <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
@@ -24798,7 +24798,7 @@
       </c>
     </row>
     <row r="17" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="99"/>
+      <c r="A17" s="121"/>
       <c r="B17" s="4" t="s">
         <v>40</v>
       </c>
@@ -24873,7 +24873,7 @@
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A18" s="97" t="s">
+      <c r="A18" s="119" t="s">
         <v>41</v>
       </c>
       <c r="B18" s="9" t="s">
@@ -24950,7 +24950,7 @@
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A19" s="98"/>
+      <c r="A19" s="120"/>
       <c r="B19" s="2" t="s">
         <v>42</v>
       </c>
@@ -25025,7 +25025,7 @@
       </c>
     </row>
     <row r="20" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="98"/>
+      <c r="A20" s="120"/>
       <c r="B20" s="4" t="s">
         <v>42</v>
       </c>
@@ -25100,7 +25100,7 @@
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A21" s="98"/>
+      <c r="A21" s="120"/>
       <c r="B21" s="9" t="s">
         <v>40</v>
       </c>
@@ -25175,7 +25175,7 @@
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A22" s="98"/>
+      <c r="A22" s="120"/>
       <c r="B22" s="2" t="s">
         <v>40</v>
       </c>
@@ -25250,7 +25250,7 @@
       </c>
     </row>
     <row r="23" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="99"/>
+      <c r="A23" s="121"/>
       <c r="B23" s="11" t="s">
         <v>40</v>
       </c>
@@ -25325,7 +25325,7 @@
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="119" t="s">
         <v>43</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -25402,7 +25402,7 @@
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A25" s="98"/>
+      <c r="A25" s="120"/>
       <c r="B25" s="2" t="s">
         <v>39</v>
       </c>
@@ -25477,7 +25477,7 @@
       </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A26" s="98"/>
+      <c r="A26" s="120"/>
       <c r="B26" s="2" t="s">
         <v>39</v>
       </c>
@@ -25552,7 +25552,7 @@
       </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A27" s="98"/>
+      <c r="A27" s="120"/>
       <c r="B27" s="2" t="s">
         <v>39</v>
       </c>
@@ -25627,7 +25627,7 @@
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A28" s="98"/>
+      <c r="A28" s="120"/>
       <c r="B28" s="2" t="s">
         <v>39</v>
       </c>
@@ -25702,7 +25702,7 @@
       </c>
     </row>
     <row r="29" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="99"/>
+      <c r="A29" s="121"/>
       <c r="B29" s="4" t="s">
         <v>39</v>
       </c>
@@ -25779,6 +25779,17 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A2:Y2"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="U4:W4"/>
+    <mergeCell ref="L3:L5"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="F3:F5"/>
     <mergeCell ref="A24:A29"/>
     <mergeCell ref="A6:A17"/>
     <mergeCell ref="A18:A23"/>
@@ -25795,17 +25806,6 @@
     <mergeCell ref="A3:B4"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="M3:N3"/>
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="U4:W4"/>
-    <mergeCell ref="L3:L5"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="F3:F5"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>